<commit_message>
Price list: AeroLouver Max Rail shows Price on request
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HCpRaxMiB3sTJWgHg1YfTk
</commit_message>
<xml_diff>
--- a/agst/shopify/aluglobus-shop-products-prices.xlsx
+++ b/agst/shopify/aluglobus-shop-products-prices.xlsx
@@ -2959,10 +2959,12 @@
           <t>https://aluglobusfence.com/shop/aluminum-fence/aerolouver-max-rail-1-5-flat-angle-l/</t>
         </is>
       </c>
-      <c r="D131" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E131" s="2" t="n"/>
+      <c r="D131" s="4" t="n"/>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>Price on request</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -3242,6 +3244,7 @@
         </is>
       </c>
     </row>
+    <row r="146"/>
     <row r="147">
       <c r="B147" s="5" t="inlineStr">
         <is>

</xml_diff>